<commit_message>
docs: update production batch planning reference
</commit_message>
<xml_diff>
--- a/参考资料/果葡糖浆生产线批次划分规则1.xlsx
+++ b/参考资料/果葡糖浆生产线批次划分规则1.xlsx
@@ -10,6 +10,7 @@
     <sheet name="批次划分规则1" sheetId="1" r:id="rId1"/>
     <sheet name="批次信息详表" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="952">
   <si>
     <t>层级</t>
   </si>
@@ -3216,13 +3217,16 @@
     <t>糖化液DE值</t>
   </si>
   <si>
-    <t>第3 层：糖化批次：成本归集、质量追溯、物理分界、上下游关联</t>
+    <t>第3 层：投料批次：成本归集、质量追溯、原料绑定、上下游关联</t>
   </si>
   <si>
     <t>编码格式： YYMMDD-W-HHMM；示例： 260810-W-0800
 说明： 投料批次覆盖拆包、溶粉、液化工序，以投料口为起点，液化液入糖化罐口阀为终点。糖化酶、糖化罐酸添加计入相应糖化罐，不在此层处理。时间窗口长度动态计算，首尾相接。</t>
   </si>
   <si>
+    <t>6、状态字段</t>
+  </si>
+  <si>
     <t>投料批次号</t>
   </si>
   <si>
@@ -3235,6 +3239,12 @@
     <t>该投料批次绑定的线边玉米淀粉批次</t>
   </si>
   <si>
+    <t>原料成本（元）</t>
+  </si>
+  <si>
+    <t>该批次投入的玉米淀粉成本</t>
+  </si>
+  <si>
     <t>该批次启动时间（系统切片起点，由DCS启动时间）</t>
   </si>
   <si>
@@ -3244,12 +3254,33 @@
     <t>该批次投入的玉米淀粉总吨数</t>
   </si>
   <si>
+    <t>液化液DE值</t>
+  </si>
+  <si>
+    <t>液化液葡萄糖值</t>
+  </si>
+  <si>
+    <t>15-20</t>
+  </si>
+  <si>
+    <t>拆包、溶粉、液化环节附加成本（元）</t>
+  </si>
+  <si>
     <t>投料开始时间</t>
   </si>
   <si>
     <t>DCS记录的投料开始时间</t>
   </si>
   <si>
+    <t>液化液浓度（°Bx）</t>
+  </si>
+  <si>
+    <t>液化液浓度</t>
+  </si>
+  <si>
+    <t>原料成本 + 附加成本</t>
+  </si>
+  <si>
     <t>设备有效容积 ÷ 批次启动时的平均流量（质量流量计）</t>
   </si>
   <si>
@@ -3259,10 +3290,19 @@
     <t>DCS记录的投料结束时间</t>
   </si>
   <si>
-    <t>该批次液化液的总产出量</t>
-  </si>
-  <si>
-    <t>3、线边批次到投料批次的关联方式</t>
+    <t>液化液pH值</t>
+  </si>
+  <si>
+    <t>5.5-6.0</t>
+  </si>
+  <si>
+    <t>该批次液化液的总产出量，淀粉乳液罐A液位达到平衡以后的淀粉乳质量流量计计量。</t>
+  </si>
+  <si>
+    <t>4、线边批次到投料批次的关联方式</t>
+  </si>
+  <si>
+    <t>过程时间与窗口规则</t>
   </si>
   <si>
     <t>线边原料批次是投料批次的上游</t>
@@ -3271,7 +3311,743 @@
     <t>投料时，操作工或系统选择当前使用的线边原料批次号，绑定到投料批次</t>
   </si>
   <si>
+    <t>去向糖化批次号</t>
+  </si>
+  <si>
+    <t>该投料批次的液化液进入哪个糖化罐</t>
+  </si>
+  <si>
+    <t>20260810-TH03-001</t>
+  </si>
+  <si>
+    <t>Tw = 投料口至糖化罐入口阀管道及设备有效容积 ÷ 淀粉乳流量（质量流量计），流量取批次启动时的平均流量</t>
+  </si>
+  <si>
     <t>数据来源</t>
+  </si>
+  <si>
+    <t>两种选择：
+1、线边工位号由WMS自动绑定第2.1层批号；
+2、线边工位号由WMS自动绑定第2.2层批号；</t>
+  </si>
+  <si>
+    <t>液化液入糖化罐阀门位号</t>
+  </si>
+  <si>
+    <t>液化液进入糖化罐的阀门位号与进料字段。进料时间。</t>
+  </si>
+  <si>
+    <t>DCS-VLV-20260810-0600；
+2026/8/10 12:00:00</t>
+  </si>
+  <si>
+    <t>第一次以DCS投料启动信号为准，过程时间预设5小时，淀粉乳液质量流量计稳定后，重新计算过程时间，后续为上一批次窗口终点（系统自动滚动）</t>
+  </si>
+  <si>
+    <t>窗口终点</t>
+  </si>
+  <si>
+    <t>当前批次启动时间 + 过程时间</t>
+  </si>
+  <si>
+    <t>以进入投料口的入口时间为准</t>
+  </si>
+  <si>
+    <t>第2 层：入厂原料批次：成本归集、库存管理、先进先出、追溯关联</t>
+  </si>
+  <si>
+    <t>编码格式： YYMMDD-序号-供应商ID号；示例： 260810-001-XXX
+说明： 入厂原料批次是玉米淀粉进入工厂后的第一批次记录，由仓储物流岗位根据车辆入厂信息创建，关联供应商批次信息。</t>
+  </si>
+  <si>
+    <t>6、入库去向的两种场景</t>
+  </si>
+  <si>
+    <t>入库去向类型</t>
+  </si>
+  <si>
+    <t>去向库位/工位号</t>
+  </si>
+  <si>
+    <t>后续关联</t>
+  </si>
+  <si>
+    <t>入厂原料批次号</t>
+  </si>
+  <si>
+    <t>260810-001-XXX</t>
+  </si>
+  <si>
+    <t>供应商批次号</t>
+  </si>
+  <si>
+    <t>供应商提供的原料批次编号</t>
+  </si>
+  <si>
+    <t>SUP-20260801-A</t>
+  </si>
+  <si>
+    <t>卸货状态</t>
+  </si>
+  <si>
+    <t>待卸货 / 卸货中 / 已卸货</t>
+  </si>
+  <si>
+    <t>原料卸货进度</t>
+  </si>
+  <si>
+    <t>卸货入平面库</t>
+  </si>
+  <si>
+    <t>平面库</t>
+  </si>
+  <si>
+    <t>K001</t>
+  </si>
+  <si>
+    <t>关联至2.1层 平面库库位批次</t>
+  </si>
+  <si>
+    <t>供应商ID号</t>
+  </si>
+  <si>
+    <t>供应商唯一标识</t>
+  </si>
+  <si>
+    <t>XXX</t>
+  </si>
+  <si>
+    <t>供应商名称</t>
+  </si>
+  <si>
+    <t>供应商全称</t>
+  </si>
+  <si>
+    <t>XX淀粉有限公司</t>
+  </si>
+  <si>
+    <t>质量状态</t>
+  </si>
+  <si>
+    <t>卸货到线边</t>
+  </si>
+  <si>
+    <t>线边</t>
+  </si>
+  <si>
+    <t>XB01</t>
+  </si>
+  <si>
+    <t>关联至2.2层 线边投料原料批次</t>
+  </si>
+  <si>
+    <t>供应商生产日期</t>
+  </si>
+  <si>
+    <t>原料的生产日期（供应商提供）</t>
+  </si>
+  <si>
+    <t>7、入库去向处理逻辑</t>
+  </si>
+  <si>
+    <t>供应商质检报告编号</t>
+  </si>
+  <si>
+    <t>供应商提供的质检报告</t>
+  </si>
+  <si>
+    <t>QA-SUP-20260801</t>
+  </si>
+  <si>
+    <t>处理方式</t>
+  </si>
+  <si>
+    <t>入厂日期</t>
+  </si>
+  <si>
+    <t>车辆入厂日期</t>
+  </si>
+  <si>
+    <t>供应商质检结论</t>
+  </si>
+  <si>
+    <t>供应商自检结论</t>
+  </si>
+  <si>
+    <t>入平面库</t>
+  </si>
+  <si>
+    <t>仓储物流人员录入“入库去向类型=平面库”、“去向库位/工位号=K001”→系统自动创建2.1层平面库库位批次，继承入厂原料批次信息</t>
+  </si>
+  <si>
+    <t>入厂时间</t>
+  </si>
+  <si>
+    <t>车辆入厂具体时间</t>
+  </si>
+  <si>
+    <t>原料生产批次（供应商端）</t>
+  </si>
+  <si>
+    <t>供应商端的生产批次标识</t>
+  </si>
+  <si>
+    <t>BATCH-20260728-01</t>
+  </si>
+  <si>
+    <t>水分（%）</t>
+  </si>
+  <si>
+    <t>原料水分含量</t>
+  </si>
+  <si>
+    <t>到线边</t>
+  </si>
+  <si>
+    <t>仓储物流人员录入“入库去向类型=线边”、“去向库位/工位号=XB01”→系统自动创建2.2层线边投料原料批次，继承入厂原料批次信息</t>
+  </si>
+  <si>
+    <t>车次序号</t>
+  </si>
+  <si>
+    <t>当天车辆入厂顺序号，从001开始递增</t>
+  </si>
+  <si>
+    <t>细度（%）</t>
+  </si>
+  <si>
+    <t>原料细度</t>
+  </si>
+  <si>
+    <t>8、成本信息</t>
+  </si>
+  <si>
+    <t>运输车辆车牌</t>
+  </si>
+  <si>
+    <t>白度</t>
+  </si>
+  <si>
+    <t>原料白度</t>
+  </si>
+  <si>
+    <t>原料名称</t>
+  </si>
+  <si>
+    <t>玉米淀粉</t>
+  </si>
+  <si>
+    <t>去向线边原料批次号</t>
+  </si>
+  <si>
+    <t>移库至线边的原料批次</t>
+  </si>
+  <si>
+    <t>20260810-001-XB01</t>
+  </si>
+  <si>
+    <t>蛋白质（%）</t>
+  </si>
+  <si>
+    <t>原料蛋白质含量</t>
+  </si>
+  <si>
+    <t>采购单价（元/吨）</t>
+  </si>
+  <si>
+    <t>该批次原料的采购单价</t>
+  </si>
+  <si>
+    <t>包装规格（kg/袋）</t>
+  </si>
+  <si>
+    <t>每袋重量</t>
+  </si>
+  <si>
+    <t>去向投料批次号</t>
+  </si>
+  <si>
+    <t>直接参与投料的批次</t>
+  </si>
+  <si>
+    <t>灰分（%）</t>
+  </si>
+  <si>
+    <t>原料灰分含量</t>
+  </si>
+  <si>
+    <t>采购总价（元）</t>
+  </si>
+  <si>
+    <t>总重量 × 采购单价</t>
+  </si>
+  <si>
+    <t>总袋数</t>
+  </si>
+  <si>
+    <t>本车总袋数</t>
+  </si>
+  <si>
+    <t>斑点（个/cm²）</t>
+  </si>
+  <si>
+    <t>原料斑点</t>
+  </si>
+  <si>
+    <t>该批次原料的运输费用</t>
+  </si>
+  <si>
+    <t>总重量（吨）</t>
+  </si>
+  <si>
+    <t>本车原料总重量（袋数×规格）</t>
+  </si>
+  <si>
+    <t>二氧化硫（ppm）</t>
+  </si>
+  <si>
+    <t>原料二氧化硫含量</t>
+  </si>
+  <si>
+    <t>≤30</t>
+  </si>
+  <si>
+    <t>其他费用（元）</t>
+  </si>
+  <si>
+    <t>装卸费、保险费等</t>
+  </si>
+  <si>
+    <t>车辆称重重量（吨）</t>
+  </si>
+  <si>
+    <t>地磅称重重量</t>
+  </si>
+  <si>
+    <t>质量检验结论</t>
+  </si>
+  <si>
+    <t>采购总价 + 运输费用 + 其他费用</t>
+  </si>
+  <si>
+    <t>磅差（吨）</t>
+  </si>
+  <si>
+    <t>称重重量 - 计算重量</t>
+  </si>
+  <si>
+    <t>总成本 ÷ 总重量</t>
+  </si>
+  <si>
+    <t>外观检验</t>
+  </si>
+  <si>
+    <t>外观是否合格</t>
+  </si>
+  <si>
+    <t>平面库 / 线边</t>
+  </si>
+  <si>
+    <t>平面库库位号或线边工位号</t>
+  </si>
+  <si>
+    <t>上游</t>
+  </si>
+  <si>
+    <t>入库时间</t>
+  </si>
+  <si>
+    <t>物料入库完成时间</t>
+  </si>
+  <si>
+    <t>原料的生产日期</t>
+  </si>
+  <si>
+    <t>仓储物流岗位取样时间</t>
+  </si>
+  <si>
+    <t>取样人</t>
+  </si>
+  <si>
+    <t>取样操作人员</t>
+  </si>
+  <si>
+    <t>下游</t>
+  </si>
+  <si>
+    <r>
+      <t>去向库位</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>工位号</t>
+    </r>
+  </si>
+  <si>
+    <t>入库去向（平面库库位或线边工位）</t>
+  </si>
+  <si>
+    <t>K001 / XB01</t>
+  </si>
+  <si>
+    <t>到货状态</t>
+  </si>
+  <si>
+    <t>已卸货</t>
+  </si>
+  <si>
+    <t>第2.1 层：平面库库位批次信息：库存管理、先进先出、追溯关联</t>
+  </si>
+  <si>
+    <t>编码格式： YYMMDD-序号-K库位号；示例： 260810-001-K001
+说明： 入厂原料卸货至平面库后，按库位划分的批次，直接关联入厂原料批次。</t>
+  </si>
+  <si>
+    <t>4、成本信息</t>
+  </si>
+  <si>
+    <t>平面库库位批次号</t>
+  </si>
+  <si>
+    <t>260810-001-K001</t>
+  </si>
+  <si>
+    <t>关联入厂原料批次号</t>
+  </si>
+  <si>
+    <t>关联的入厂批次</t>
+  </si>
+  <si>
+    <t>来源入厂批次总成本（元）</t>
+  </si>
+  <si>
+    <t>关联的入厂原料批次总成本</t>
+  </si>
+  <si>
+    <t>入库重量（吨）</t>
+  </si>
+  <si>
+    <t>该库位批次入库重量</t>
+  </si>
+  <si>
+    <t>库位号</t>
+  </si>
+  <si>
+    <t>平面库具体库位编号</t>
+  </si>
+  <si>
+    <t>来源入厂批次总成本 ÷ 入库重量</t>
+  </si>
+  <si>
+    <t>入库叉车编号</t>
+  </si>
+  <si>
+    <t>执行入库操作的叉车</t>
+  </si>
+  <si>
+    <t>FC-01</t>
+  </si>
+  <si>
+    <t>移库出库重量（吨）</t>
+  </si>
+  <si>
+    <t>已移库至线边的重量</t>
+  </si>
+  <si>
+    <t>物料入库时间</t>
+  </si>
+  <si>
+    <t>260810-001-XB01</t>
+  </si>
+  <si>
+    <t>移库出库成本（元）</t>
+  </si>
+  <si>
+    <t>移库出库重量 × 单位成本</t>
+  </si>
+  <si>
+    <t>入库袋数</t>
+  </si>
+  <si>
+    <t>入库总袋数</t>
+  </si>
+  <si>
+    <t>当前库存重量（吨）</t>
+  </si>
+  <si>
+    <t>该库位批次剩余重量</t>
+  </si>
+  <si>
+    <t>入库总重量</t>
+  </si>
+  <si>
+    <t>当前库存成本（元）</t>
+  </si>
+  <si>
+    <t>当前库存重量 × 单位成本</t>
+  </si>
+  <si>
+    <t>当前库存袋数</t>
+  </si>
+  <si>
+    <t>当前剩余袋数</t>
+  </si>
+  <si>
+    <t>当前剩余重量</t>
+  </si>
+  <si>
+    <t>第2.2层：线边工位批次信息：投料准备、成本传递、追溯关联</t>
+  </si>
+  <si>
+    <t>编码格式： YYMMDD-序号-XB线边工位号；示例： 20260810-001-XB01
+说明： 平面库物料移库至生产线边工位后生成的批次，关联平面库库位批次，是投料批次的上游来源。</t>
+  </si>
+  <si>
+    <t>线边原料批次号</t>
+  </si>
+  <si>
+    <t>来源平面库批次总成本（元）</t>
+  </si>
+  <si>
+    <t>关联的平面库库位批次总成本</t>
+  </si>
+  <si>
+    <t>关联平面库库位批次号</t>
+  </si>
+  <si>
+    <t>关联的库位批次</t>
+  </si>
+  <si>
+    <t>20260810-001-K001</t>
+  </si>
+  <si>
+    <t>移库重量（吨）</t>
+  </si>
+  <si>
+    <t>该线边批次移库重量</t>
+  </si>
+  <si>
+    <t>20260810-001-XXX</t>
+  </si>
+  <si>
+    <t>来源平面库批次总成本 ÷ 移库重量</t>
+  </si>
+  <si>
+    <t>线边工位号</t>
+  </si>
+  <si>
+    <t>生产线边工位编号</t>
+  </si>
+  <si>
+    <t>投料消耗重量（吨）</t>
+  </si>
+  <si>
+    <t>已投料消耗的重量</t>
+  </si>
+  <si>
+    <t>移库叉车编号</t>
+  </si>
+  <si>
+    <t>执行移库操作的叉车</t>
+  </si>
+  <si>
+    <t>FC-02</t>
+  </si>
+  <si>
+    <t>该线边原料参与哪些投料批次</t>
+  </si>
+  <si>
+    <t>投料消耗成本（元）</t>
+  </si>
+  <si>
+    <t>投料消耗重量 × 单位成本</t>
+  </si>
+  <si>
+    <t>移库时间</t>
+  </si>
+  <si>
+    <t>物料移至线边的时间</t>
+  </si>
+  <si>
+    <t>投料消耗量（吨）</t>
+  </si>
+  <si>
+    <t>线边剩余重量（吨）</t>
+  </si>
+  <si>
+    <t>线边当前剩余重量</t>
+  </si>
+  <si>
+    <t>移库袋数</t>
+  </si>
+  <si>
+    <t>移库总袋数</t>
+  </si>
+  <si>
+    <t>剩余重量（吨）</t>
+  </si>
+  <si>
+    <t>线边剩余未投料重量</t>
+  </si>
+  <si>
+    <t>线边剩余成本（元）</t>
+  </si>
+  <si>
+    <t>线边剩余重量 × 单位成本</t>
+  </si>
+  <si>
+    <t>各层级成本信息汇总</t>
+  </si>
+  <si>
+    <t>总成本构成</t>
+  </si>
+  <si>
+    <t>单位成本计算</t>
+  </si>
+  <si>
+    <t>当前库存总成本</t>
+  </si>
+  <si>
+    <t>第2层 入厂原料批次</t>
+  </si>
+  <si>
+    <t>第2.1层 平面库库位批次</t>
+  </si>
+  <si>
+    <t>来源入厂批次总成本（按入库重量继承）</t>
+  </si>
+  <si>
+    <t>第2.2层 线边投料原料批次</t>
+  </si>
+  <si>
+    <t>来源平面库批次总成本（按移库重量继承）</t>
+  </si>
+  <si>
+    <t>第1层：供应商信息：质量追溯起点、入厂关联、供应商评估</t>
+  </si>
+  <si>
+    <t>供应商原料批次
+供应商自行划分，并提供原料出厂数据（包装规格、质量数据、生产日期）
+编号说明：印刷在袋子上、纸质单子（包括供应商名称、规格、质检数据、生产日期等）。</t>
+  </si>
+  <si>
+    <t>2、供应商质量信息</t>
+  </si>
+  <si>
+    <t>3、关联字段</t>
+  </si>
+  <si>
+    <t>供应商提供的批次编号（印刷在袋子上或纸质单子）</t>
+  </si>
+  <si>
+    <t>供应商检测的水分含量</t>
+  </si>
+  <si>
+    <t>该供应商批次对应的入厂批次</t>
+  </si>
+  <si>
+    <t>数据状态</t>
+  </si>
+  <si>
+    <t>待录入 / 已录入 / 已确认</t>
+  </si>
+  <si>
+    <t>数据录入状态</t>
+  </si>
+  <si>
+    <t>供应商检测的细度</t>
+  </si>
+  <si>
+    <t>供应商代码</t>
+  </si>
+  <si>
+    <t>供应商唯一编码（系统内）</t>
+  </si>
+  <si>
+    <t>S-001</t>
+  </si>
+  <si>
+    <t>供应商检测的白度</t>
+  </si>
+  <si>
+    <t>供应商检测的蛋白质含量</t>
+  </si>
+  <si>
+    <t>原料规格</t>
+  </si>
+  <si>
+    <t>原料等级/规格</t>
+  </si>
+  <si>
+    <t>一级品</t>
+  </si>
+  <si>
+    <t>供应商检测的灰分含量</t>
+  </si>
+  <si>
+    <t>生产日期</t>
+  </si>
+  <si>
+    <t>原料生产日期（供应商提供）</t>
+  </si>
+  <si>
+    <t>供应商检测的斑点</t>
+  </si>
+  <si>
+    <t>保质期</t>
+  </si>
+  <si>
+    <t>原料保质期</t>
+  </si>
+  <si>
+    <t>12个月</t>
+  </si>
+  <si>
+    <t>供应商检测的二氧化硫含量</t>
+  </si>
+  <si>
+    <t>本批次总袋数</t>
+  </si>
+  <si>
+    <t>供应商提供的质检报告编号</t>
+  </si>
+  <si>
+    <t>本批次原料总重量</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">费用池：公共成本月底分摊到批次，对批次成本进行修正，最后汇总归集。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>公共成本归集</t>
+    </r>
+  </si>
+  <si>
+    <t>人力成本预设，月底根据最终支出修正批次成本，最后汇总归集。</t>
   </si>
   <si>
     <t>字段 说明 示例
@@ -3296,7 +4072,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="48">
+  <fonts count="51">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3432,6 +4208,20 @@
     <font>
       <sz val="12"/>
       <color rgb="FFC00000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="var(--dsw-font-markdown-table)"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -3608,15 +4398,23 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10.5"/>
-      <color rgb="FF0F1115"/>
-      <name val="var(--ds-font-family-code)"/>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFC00000"/>
+      <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FFC00000"/>
       <name val="Songti SC Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF0F1115"/>
+      <name val="var(--ds-font-family-code)"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3632,7 +4430,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3666,6 +4464,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3868,7 +4672,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -4006,6 +4810,17 @@
     </border>
     <border>
       <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -4122,137 +4937,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="12" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4685,19 +5500,106 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4718,13 +5620,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4736,10 +5638,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -4754,10 +5656,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5296,304 +6198,304 @@
   </cols>
   <sheetData>
     <row r="2" ht="42" customHeight="1" spans="1:6">
-      <c r="A2" s="146" t="s">
+      <c r="A2" s="175" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="146" t="s">
+      <c r="B2" s="175" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="146" t="s">
+      <c r="C2" s="175" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="146" t="s">
+      <c r="D2" s="175" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="146" t="s">
+      <c r="E2" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="146" t="s">
+      <c r="F2" s="175" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" s="145" customFormat="1" ht="68" customHeight="1" spans="1:6">
-      <c r="A3" s="147" t="s">
+    <row r="3" s="174" customFormat="1" ht="68" customHeight="1" spans="1:6">
+      <c r="A3" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="147" t="s">
+      <c r="B3" s="176" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="148" t="s">
+      <c r="C3" s="177" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="147" t="s">
+      <c r="D3" s="176" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="147" t="s">
+      <c r="E3" s="176" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="148" t="s">
+      <c r="F3" s="177" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" s="145" customFormat="1" ht="78" customHeight="1" spans="1:6">
-      <c r="A4" s="148" t="s">
+    <row r="4" s="174" customFormat="1" ht="78" customHeight="1" spans="1:6">
+      <c r="A4" s="177" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="148"/>
-      <c r="C4" s="148"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
-      <c r="F4" s="148"/>
-    </row>
-    <row r="5" s="145" customFormat="1" ht="66" customHeight="1" spans="1:6">
-      <c r="A5" s="149" t="s">
+      <c r="B4" s="177"/>
+      <c r="C4" s="177"/>
+      <c r="D4" s="177"/>
+      <c r="E4" s="177"/>
+      <c r="F4" s="177"/>
+    </row>
+    <row r="5" s="174" customFormat="1" ht="66" customHeight="1" spans="1:6">
+      <c r="A5" s="178" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="149" t="s">
+      <c r="B5" s="178" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="150" t="s">
+      <c r="C5" s="179" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="151" t="s">
+      <c r="D5" s="180" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="151" t="s">
+      <c r="E5" s="180" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="150" t="s">
+      <c r="F5" s="179" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" s="145" customFormat="1" ht="57" customHeight="1" spans="1:6">
-      <c r="A6" s="152">
+    <row r="6" s="174" customFormat="1" ht="57" customHeight="1" spans="1:6">
+      <c r="A6" s="181">
         <v>2.1</v>
       </c>
-      <c r="B6" s="152" t="s">
+      <c r="B6" s="181" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="153" t="s">
+      <c r="C6" s="182" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="154" t="s">
+      <c r="D6" s="183" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="154" t="s">
+      <c r="E6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="153" t="s">
+      <c r="F6" s="182" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" s="145" customFormat="1" ht="50" customHeight="1" spans="1:6">
-      <c r="A7" s="152">
+    <row r="7" s="174" customFormat="1" ht="50" customHeight="1" spans="1:6">
+      <c r="A7" s="181">
         <v>2.2</v>
       </c>
-      <c r="B7" s="152" t="s">
+      <c r="B7" s="181" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="153" t="s">
+      <c r="C7" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="154" t="s">
+      <c r="D7" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="154" t="s">
+      <c r="E7" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="153" t="s">
+      <c r="F7" s="182" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" ht="67" customHeight="1" spans="1:6">
-      <c r="A8" s="152" t="s">
+      <c r="A8" s="181" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="152" t="s">
+      <c r="B8" s="181" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="153" t="s">
+      <c r="C8" s="182" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="154" t="s">
+      <c r="D8" s="183" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="154" t="s">
+      <c r="E8" s="183" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="155" t="s">
+      <c r="F8" s="184" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" ht="54" customHeight="1" spans="1:6">
-      <c r="A9" s="152" t="s">
+      <c r="A9" s="181" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="152" t="s">
+      <c r="B9" s="181" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="156" t="s">
+      <c r="C9" s="185" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="154" t="s">
+      <c r="D9" s="183" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="154" t="s">
+      <c r="E9" s="183" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="155" t="s">
+      <c r="F9" s="184" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1" spans="1:6">
-      <c r="A10" s="152" t="s">
+      <c r="A10" s="181" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="154" t="s">
+      <c r="B10" s="183" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="156" t="s">
+      <c r="C10" s="185" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="154" t="s">
+      <c r="D10" s="183" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="154" t="s">
+      <c r="E10" s="183" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="155" t="s">
+      <c r="F10" s="184" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1" spans="1:6">
-      <c r="A11" s="152" t="s">
+      <c r="A11" s="181" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="152" t="s">
+      <c r="B11" s="181" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="153" t="s">
+      <c r="C11" s="182" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="154" t="s">
+      <c r="D11" s="183" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="154" t="s">
+      <c r="E11" s="183" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="155" t="s">
+      <c r="F11" s="184" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1" spans="1:6">
-      <c r="A12" s="152" t="s">
+      <c r="A12" s="181" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="154" t="s">
+      <c r="B12" s="183" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="153" t="s">
+      <c r="C12" s="182" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="154" t="s">
+      <c r="D12" s="183" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="154" t="s">
+      <c r="E12" s="183" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="155" t="s">
+      <c r="F12" s="184" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="13" ht="43" customHeight="1" spans="1:6">
-      <c r="A13" s="152" t="s">
+      <c r="A13" s="181" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="154" t="s">
+      <c r="B13" s="183" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="156" t="s">
+      <c r="C13" s="185" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="154" t="s">
+      <c r="D13" s="183" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="154" t="s">
+      <c r="E13" s="183" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="155" t="s">
+      <c r="F13" s="184" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="14" ht="51" customHeight="1" spans="1:6">
-      <c r="A14" s="152" t="s">
+      <c r="A14" s="181" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="152" t="s">
+      <c r="B14" s="181" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="153" t="s">
+      <c r="C14" s="182" t="s">
         <v>66</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="183" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="154" t="s">
+      <c r="E14" s="183" t="s">
         <v>68</v>
       </c>
-      <c r="F14" s="155" t="s">
+      <c r="F14" s="184" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="15" ht="65" customHeight="1" spans="1:6">
-      <c r="A15" s="149" t="s">
+      <c r="A15" s="178" t="s">
         <v>70</v>
       </c>
-      <c r="B15" s="149" t="s">
+      <c r="B15" s="178" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="150" t="s">
+      <c r="C15" s="179" t="s">
         <v>72</v>
       </c>
-      <c r="D15" s="151" t="s">
+      <c r="D15" s="180" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="151" t="s">
+      <c r="E15" s="180" t="s">
         <v>74</v>
       </c>
-      <c r="F15" s="157" t="s">
+      <c r="F15" s="186" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="16" ht="35" customHeight="1" spans="1:6">
-      <c r="A16" s="158"/>
-      <c r="B16" s="158"/>
-      <c r="C16" s="159"/>
-      <c r="D16" s="160"/>
-      <c r="E16" s="160"/>
-      <c r="F16" s="161"/>
+      <c r="A16" s="187"/>
+      <c r="B16" s="187"/>
+      <c r="C16" s="188"/>
+      <c r="D16" s="189"/>
+      <c r="E16" s="189"/>
+      <c r="F16" s="190"/>
     </row>
     <row r="17" customHeight="1" spans="1:6">
-      <c r="A17" s="162" t="s">
+      <c r="A17" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="162"/>
-      <c r="C17" s="162"/>
-      <c r="D17" s="162"/>
-      <c r="E17" s="162"/>
-      <c r="F17" s="162"/>
+      <c r="B17" s="191"/>
+      <c r="C17" s="191"/>
+      <c r="D17" s="191"/>
+      <c r="E17" s="191"/>
+      <c r="F17" s="191"/>
     </row>
     <row r="18" customHeight="1" spans="1:6">
-      <c r="A18" s="163"/>
-      <c r="B18" s="164" t="s">
+      <c r="A18" s="192"/>
+      <c r="B18" s="193" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="164" t="s">
+      <c r="C18" s="193" t="s">
         <v>78</v>
       </c>
-      <c r="D18" s="164"/>
-      <c r="E18" s="164"/>
-      <c r="F18" s="164" t="s">
+      <c r="D18" s="193"/>
+      <c r="E18" s="193"/>
+      <c r="F18" s="193" t="s">
         <v>5</v>
       </c>
     </row>
@@ -5609,7 +6511,7 @@
       </c>
       <c r="D19" s="112"/>
       <c r="E19" s="112"/>
-      <c r="F19" s="165" t="s">
+      <c r="F19" s="194" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5625,7 +6527,7 @@
       </c>
       <c r="D20" s="112"/>
       <c r="E20" s="112"/>
-      <c r="F20" s="166"/>
+      <c r="F20" s="195"/>
     </row>
     <row r="21" customHeight="1" spans="1:6">
       <c r="A21" s="79">
@@ -5639,7 +6541,7 @@
       </c>
       <c r="D21" s="112"/>
       <c r="E21" s="112"/>
-      <c r="F21" s="166"/>
+      <c r="F21" s="195"/>
     </row>
     <row r="22" customHeight="1" spans="1:6">
       <c r="A22" s="79">
@@ -5653,7 +6555,7 @@
       </c>
       <c r="D22" s="112"/>
       <c r="E22" s="112"/>
-      <c r="F22" s="166"/>
+      <c r="F22" s="195"/>
     </row>
     <row r="23" customHeight="1" spans="1:6">
       <c r="A23" s="5"/>
@@ -5664,46 +6566,46 @@
       <c r="F23" s="5"/>
     </row>
     <row r="24" customHeight="1" spans="1:6">
-      <c r="A24" s="167" t="s">
+      <c r="A24" s="196" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="168"/>
-      <c r="C24" s="168"/>
-      <c r="D24" s="168"/>
-      <c r="E24" s="168"/>
-      <c r="F24" s="168"/>
+      <c r="B24" s="197"/>
+      <c r="C24" s="197"/>
+      <c r="D24" s="197"/>
+      <c r="E24" s="197"/>
+      <c r="F24" s="197"/>
     </row>
     <row r="25" customHeight="1" spans="1:6">
-      <c r="A25" s="168"/>
-      <c r="B25" s="168"/>
-      <c r="C25" s="168"/>
-      <c r="D25" s="168"/>
-      <c r="E25" s="168"/>
-      <c r="F25" s="168"/>
+      <c r="A25" s="197"/>
+      <c r="B25" s="197"/>
+      <c r="C25" s="197"/>
+      <c r="D25" s="197"/>
+      <c r="E25" s="197"/>
+      <c r="F25" s="197"/>
     </row>
     <row r="26" customHeight="1" spans="1:6">
-      <c r="A26" s="168"/>
-      <c r="B26" s="168"/>
-      <c r="C26" s="168"/>
-      <c r="D26" s="168"/>
-      <c r="E26" s="168"/>
-      <c r="F26" s="168"/>
+      <c r="A26" s="197"/>
+      <c r="B26" s="197"/>
+      <c r="C26" s="197"/>
+      <c r="D26" s="197"/>
+      <c r="E26" s="197"/>
+      <c r="F26" s="197"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:6">
-      <c r="A27" s="168"/>
-      <c r="B27" s="168"/>
-      <c r="C27" s="168"/>
-      <c r="D27" s="168"/>
-      <c r="E27" s="168"/>
-      <c r="F27" s="168"/>
+      <c r="A27" s="197"/>
+      <c r="B27" s="197"/>
+      <c r="C27" s="197"/>
+      <c r="D27" s="197"/>
+      <c r="E27" s="197"/>
+      <c r="F27" s="197"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:6">
-      <c r="A28" s="168"/>
-      <c r="B28" s="168"/>
-      <c r="C28" s="168"/>
-      <c r="D28" s="168"/>
-      <c r="E28" s="168"/>
-      <c r="F28" s="168"/>
+      <c r="A28" s="197"/>
+      <c r="B28" s="197"/>
+      <c r="C28" s="197"/>
+      <c r="D28" s="197"/>
+      <c r="E28" s="197"/>
+      <c r="F28" s="197"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -5725,7 +6627,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:AB148"/>
+  <dimension ref="B1:AB207"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="1.75961538461538" customWidth="1"/>
@@ -9884,6 +10786,21 @@
       </c>
       <c r="G114" s="51"/>
       <c r="H114" s="51"/>
+      <c r="J114" s="51" t="s">
+        <v>265</v>
+      </c>
+      <c r="K114" s="51"/>
+      <c r="L114" s="51"/>
+      <c r="N114" s="51" t="s">
+        <v>197</v>
+      </c>
+      <c r="O114" s="51"/>
+      <c r="P114" s="51"/>
+      <c r="R114" s="51" t="s">
+        <v>690</v>
+      </c>
+      <c r="S114" s="51"/>
+      <c r="T114" s="51"/>
     </row>
     <row r="115" s="5" customFormat="1" ht="18" spans="2:24">
       <c r="B115" s="1" t="s">
@@ -9904,45 +10821,126 @@
       <c r="H115" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="J115" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K115" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L115" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N115" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O115" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P115" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="R115" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S115" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="T115" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="116" s="5" customFormat="1" ht="54" customHeight="1" spans="2:24">
       <c r="B116" s="41" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C116" s="41" t="s">
         <v>99</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F116" s="41" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="G116" s="41" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="117" s="5" customFormat="1" ht="53" spans="2:24">
+      <c r="J116" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="K116" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="L116" s="3">
+        <v>46244.4791666667</v>
+      </c>
+      <c r="N116" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="O116" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="P116" s="144">
+        <v>320000</v>
+      </c>
+      <c r="R116" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="S116" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="T116" s="2" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="117" s="5" customFormat="1" ht="71" spans="2:24">
       <c r="B117" s="41" t="s">
         <v>386</v>
       </c>
       <c r="C117" s="41" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="D117" s="3">
         <v>46244.3333333333</v>
       </c>
       <c r="F117" s="41" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="G117" s="41" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="H117" s="2">
         <v>100</v>
+      </c>
+      <c r="J117" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="K117" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="L117" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="N117" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="O117" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="P117" s="144">
+        <v>18000</v>
+      </c>
+      <c r="R117" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="S117" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="T117" s="2" t="s">
+        <v>485</v>
       </c>
     </row>
     <row r="118" s="5" customFormat="1" ht="53" spans="2:24">
@@ -9956,13 +10954,31 @@
         <v>46244.5</v>
       </c>
       <c r="F118" s="41" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="G118" s="41" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="H118" s="3">
         <v>46244.3333333333</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="K118" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="L118" s="2">
+        <v>30</v>
+      </c>
+      <c r="N118" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="O118" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="P118" s="144">
+        <v>338000</v>
       </c>
     </row>
     <row r="119" s="5" customFormat="1" ht="71" spans="2:24">
@@ -9970,89 +10986,2224 @@
         <v>584</v>
       </c>
       <c r="C119" s="41" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="D119" s="2">
         <v>4</v>
       </c>
       <c r="F119" s="41" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="G119" s="41" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
       <c r="H119" s="3">
         <v>46244.3541666667</v>
       </c>
-    </row>
-    <row r="120" s="5" customFormat="1" ht="45" customHeight="1" spans="2:24">
+      <c r="J119" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="K119" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="L119" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="N119" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="O119" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="P119" s="144">
+        <v>3380</v>
+      </c>
+    </row>
+    <row r="120" s="5" customFormat="1" ht="110" customHeight="1" spans="2:24">
       <c r="B120" s="41" t="s">
         <v>405</v>
       </c>
       <c r="C120" s="41" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="D120" s="2">
         <v>100</v>
       </c>
-      <c r="F120" s="135" t="s">
-        <v>703</v>
-      </c>
-      <c r="G120" s="135"/>
-      <c r="H120" s="135"/>
+      <c r="J120" s="145" t="s">
+        <v>128</v>
+      </c>
+      <c r="K120" s="145" t="s">
+        <v>129</v>
+      </c>
+      <c r="L120" s="145" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="121" s="5" customFormat="1" ht="23" customHeight="1" spans="2:24">
-      <c r="F121" s="91" t="s">
+      <c r="B121" s="135" t="s">
+        <v>715</v>
+      </c>
+      <c r="C121" s="135"/>
+      <c r="D121" s="135"/>
+      <c r="F121" s="61" t="s">
+        <v>518</v>
+      </c>
+      <c r="G121" s="61"/>
+      <c r="H121" s="61"/>
+      <c r="J121" s="61" t="s">
+        <v>716</v>
+      </c>
+      <c r="K121" s="61"/>
+      <c r="L121" s="61"/>
+      <c r="M121" s="61"/>
+      <c r="N121" s="61"/>
+      <c r="O121" s="61"/>
+      <c r="P121" s="61"/>
+    </row>
+    <row r="122" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="B122" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="G121" s="92" t="s">
+      <c r="C122" s="121" t="s">
         <v>5</v>
       </c>
-      <c r="H121" s="144"/>
-    </row>
-    <row r="122" s="5" customFormat="1" ht="36" spans="2:24">
-      <c r="F122" s="41" t="s">
-        <v>704</v>
-      </c>
-      <c r="G122" s="133" t="s">
-        <v>705</v>
-      </c>
-      <c r="H122" s="133"/>
-    </row>
-    <row r="123" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="D122" s="121"/>
+      <c r="F122" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J122" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="K122" s="121" t="s">
+        <v>597</v>
+      </c>
+      <c r="L122" s="121"/>
+      <c r="M122" s="121"/>
+      <c r="N122" s="121"/>
+      <c r="O122" s="121"/>
+      <c r="P122" s="121"/>
+    </row>
+    <row r="123" s="5" customFormat="1" ht="53" customHeight="1" spans="2:24">
+      <c r="B123" s="41" t="s">
+        <v>717</v>
+      </c>
+      <c r="C123" s="42" t="s">
+        <v>718</v>
+      </c>
+      <c r="D123" s="42"/>
       <c r="F123" s="41" t="s">
-        <v>706</v>
-      </c>
-      <c r="G123" s="42"/>
-      <c r="H123" s="42"/>
-    </row>
-    <row r="124" s="5" customFormat="1" ht="17.6"/>
-    <row r="125" s="5" customFormat="1" ht="17.6"/>
-    <row r="126" s="5" customFormat="1" ht="17.6"/>
-    <row r="127" s="5" customFormat="1" ht="17.6"/>
-    <row r="128" s="5" customFormat="1" ht="17.6"/>
-    <row r="129" s="5" customFormat="1" ht="17.6"/>
-    <row r="130" s="5" customFormat="1" ht="17.6"/>
-    <row r="131" s="5" customFormat="1" ht="17.6"/>
-    <row r="132" s="5" customFormat="1" ht="17.6"/>
-    <row r="133" s="5" customFormat="1" ht="17.6"/>
-    <row r="134" s="5" customFormat="1" ht="17.6"/>
-    <row r="135" s="5" customFormat="1" ht="17.6"/>
-    <row r="136" s="5" customFormat="1" ht="17.6"/>
-    <row r="137" s="5" customFormat="1" ht="17.6"/>
-    <row r="138" s="5" customFormat="1" ht="17.6"/>
-    <row r="139" s="5" customFormat="1" ht="17.6"/>
-    <row r="140" s="5" customFormat="1" ht="17.6"/>
-    <row r="141" s="5" customFormat="1" ht="17.6"/>
-    <row r="142" s="5" customFormat="1" ht="17.6"/>
-    <row r="143" s="5" customFormat="1" ht="17.6"/>
-    <row r="144" s="5" customFormat="1" ht="17.6"/>
-    <row r="145" s="5" customFormat="1" ht="17.6"/>
-    <row r="146" s="5" customFormat="1" ht="17.6"/>
-    <row r="147" s="5" customFormat="1" ht="17.6"/>
-    <row r="148" s="5" customFormat="1" ht="17.6"/>
+        <v>719</v>
+      </c>
+      <c r="G123" s="41" t="s">
+        <v>720</v>
+      </c>
+      <c r="H123" s="41" t="s">
+        <v>721</v>
+      </c>
+      <c r="J123" s="41" t="s">
+        <v>604</v>
+      </c>
+      <c r="K123" s="42" t="s">
+        <v>722</v>
+      </c>
+      <c r="L123" s="42"/>
+      <c r="M123" s="42"/>
+      <c r="N123" s="42"/>
+      <c r="O123" s="42"/>
+      <c r="P123" s="42"/>
+    </row>
+    <row r="124" s="5" customFormat="1" ht="108" customHeight="1" spans="2:24">
+      <c r="B124" s="146" t="s">
+        <v>723</v>
+      </c>
+      <c r="C124" s="42" t="s">
+        <v>724</v>
+      </c>
+      <c r="D124" s="42"/>
+      <c r="F124" s="41" t="s">
+        <v>725</v>
+      </c>
+      <c r="G124" s="41" t="s">
+        <v>726</v>
+      </c>
+      <c r="H124" s="147" t="s">
+        <v>727</v>
+      </c>
+      <c r="J124" s="41" t="s">
+        <v>605</v>
+      </c>
+      <c r="K124" s="42" t="s">
+        <v>728</v>
+      </c>
+      <c r="L124" s="42"/>
+      <c r="M124" s="42"/>
+      <c r="N124" s="42"/>
+      <c r="O124" s="42"/>
+      <c r="P124" s="42"/>
+    </row>
+    <row r="125" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="J125" s="41" t="s">
+        <v>729</v>
+      </c>
+      <c r="K125" s="42" t="s">
+        <v>730</v>
+      </c>
+      <c r="L125" s="42"/>
+      <c r="M125" s="42"/>
+      <c r="N125" s="42"/>
+      <c r="O125" s="42"/>
+      <c r="P125" s="42"/>
+    </row>
+    <row r="126" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="J126" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="K126" s="42" t="s">
+        <v>731</v>
+      </c>
+      <c r="L126" s="42"/>
+      <c r="M126" s="42"/>
+      <c r="N126" s="42"/>
+      <c r="O126" s="42"/>
+      <c r="P126" s="42"/>
+    </row>
+    <row r="127" s="5" customFormat="1" ht="11" customHeight="1"/>
+    <row r="128" s="5" customFormat="1" ht="36" customHeight="1" spans="2:24">
+      <c r="B128" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="C128" s="6"/>
+      <c r="D128" s="6"/>
+      <c r="E128" s="6"/>
+      <c r="F128" s="6"/>
+      <c r="G128" s="6"/>
+      <c r="H128" s="6"/>
+      <c r="I128" s="6"/>
+      <c r="J128" s="6"/>
+      <c r="K128" s="6"/>
+      <c r="L128" s="6"/>
+      <c r="M128" s="6"/>
+      <c r="N128" s="6"/>
+      <c r="O128" s="6"/>
+      <c r="P128" s="6"/>
+      <c r="Q128" s="6"/>
+      <c r="R128" s="6"/>
+      <c r="S128" s="33"/>
+      <c r="T128" s="33"/>
+      <c r="U128" s="33"/>
+      <c r="V128" s="33"/>
+      <c r="W128" s="33"/>
+      <c r="X128" s="33"/>
+    </row>
+    <row r="129" s="5" customFormat="1" ht="48" customHeight="1" spans="2:24">
+      <c r="B129" s="48" t="s">
+        <v>733</v>
+      </c>
+      <c r="C129" s="48"/>
+      <c r="D129" s="48"/>
+      <c r="E129" s="48"/>
+      <c r="F129" s="48"/>
+      <c r="G129" s="48"/>
+      <c r="H129" s="48"/>
+      <c r="I129" s="48"/>
+      <c r="J129" s="48"/>
+      <c r="K129" s="48"/>
+      <c r="L129" s="48"/>
+      <c r="M129" s="48"/>
+      <c r="N129" s="48"/>
+      <c r="O129" s="48"/>
+      <c r="P129" s="48"/>
+      <c r="Q129" s="48"/>
+      <c r="R129" s="48"/>
+      <c r="S129" s="126"/>
+      <c r="T129" s="126"/>
+      <c r="U129" s="126"/>
+      <c r="V129" s="126"/>
+      <c r="W129" s="126"/>
+      <c r="X129" s="126"/>
+    </row>
+    <row r="130" s="5" customFormat="1" ht="20.4" spans="2:24">
+      <c r="B130" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C130" s="51"/>
+      <c r="D130" s="51"/>
+      <c r="F130" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="G130" s="51"/>
+      <c r="H130" s="51"/>
+      <c r="J130" s="51" t="s">
+        <v>344</v>
+      </c>
+      <c r="K130" s="51"/>
+      <c r="L130" s="51"/>
+      <c r="N130" s="148" t="s">
+        <v>734</v>
+      </c>
+      <c r="O130" s="148"/>
+      <c r="P130" s="148"/>
+      <c r="Q130" s="148"/>
+      <c r="R130" s="148"/>
+    </row>
+    <row r="131" s="5" customFormat="1" ht="44" customHeight="1" spans="2:24">
+      <c r="B131" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H131" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J131" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K131" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L131" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N131" s="122" t="s">
+        <v>316</v>
+      </c>
+      <c r="O131" s="122" t="s">
+        <v>735</v>
+      </c>
+      <c r="P131" s="122" t="s">
+        <v>736</v>
+      </c>
+      <c r="Q131" s="123" t="s">
+        <v>737</v>
+      </c>
+      <c r="R131" s="123"/>
+    </row>
+    <row r="132" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B132" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="F132" s="119" t="s">
+        <v>740</v>
+      </c>
+      <c r="G132" s="119" t="s">
+        <v>741</v>
+      </c>
+      <c r="H132" s="119" t="s">
+        <v>742</v>
+      </c>
+      <c r="J132" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="K132" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="L132" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="N132" s="119" t="s">
+        <v>746</v>
+      </c>
+      <c r="O132" s="119" t="s">
+        <v>747</v>
+      </c>
+      <c r="P132" s="119" t="s">
+        <v>748</v>
+      </c>
+      <c r="Q132" s="99" t="s">
+        <v>749</v>
+      </c>
+      <c r="R132" s="99"/>
+    </row>
+    <row r="133" s="5" customFormat="1" ht="53" spans="2:24">
+      <c r="B133" s="2" t="s">
+        <v>750</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>752</v>
+      </c>
+      <c r="F133" s="119" t="s">
+        <v>753</v>
+      </c>
+      <c r="G133" s="119" t="s">
+        <v>754</v>
+      </c>
+      <c r="H133" s="119" t="s">
+        <v>755</v>
+      </c>
+      <c r="J133" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="K133" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="L133" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="N133" s="119" t="s">
+        <v>757</v>
+      </c>
+      <c r="O133" s="119" t="s">
+        <v>758</v>
+      </c>
+      <c r="P133" s="119" t="s">
+        <v>759</v>
+      </c>
+      <c r="Q133" s="99" t="s">
+        <v>760</v>
+      </c>
+      <c r="R133" s="99"/>
+    </row>
+    <row r="134" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B134" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="F134" s="119" t="s">
+        <v>761</v>
+      </c>
+      <c r="G134" s="119" t="s">
+        <v>762</v>
+      </c>
+      <c r="H134" s="149">
+        <v>46231</v>
+      </c>
+      <c r="J134" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="K134" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="L134" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="N134" s="148" t="s">
+        <v>763</v>
+      </c>
+      <c r="O134" s="148"/>
+      <c r="P134" s="148"/>
+      <c r="Q134" s="148"/>
+      <c r="R134" s="148"/>
+    </row>
+    <row r="135" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B135" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>741</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="F135" s="119" t="s">
+        <v>764</v>
+      </c>
+      <c r="G135" s="119" t="s">
+        <v>765</v>
+      </c>
+      <c r="H135" s="119" t="s">
+        <v>766</v>
+      </c>
+      <c r="J135" s="51" t="s">
+        <v>94</v>
+      </c>
+      <c r="K135" s="51"/>
+      <c r="L135" s="51"/>
+      <c r="N135" s="121" t="s">
+        <v>316</v>
+      </c>
+      <c r="O135" s="121" t="s">
+        <v>767</v>
+      </c>
+      <c r="P135" s="121"/>
+      <c r="Q135" s="121"/>
+      <c r="R135" s="121"/>
+    </row>
+    <row r="136" s="5" customFormat="1" ht="56" customHeight="1" spans="2:24">
+      <c r="B136" s="2" t="s">
+        <v>768</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="D136" s="150">
+        <v>46244</v>
+      </c>
+      <c r="F136" s="119" t="s">
+        <v>770</v>
+      </c>
+      <c r="G136" s="119" t="s">
+        <v>771</v>
+      </c>
+      <c r="H136" s="119" t="s">
+        <v>130</v>
+      </c>
+      <c r="J136" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K136" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L136" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N136" s="41" t="s">
+        <v>772</v>
+      </c>
+      <c r="O136" s="42" t="s">
+        <v>773</v>
+      </c>
+      <c r="P136" s="42"/>
+      <c r="Q136" s="42"/>
+      <c r="R136" s="42"/>
+    </row>
+    <row r="137" s="5" customFormat="1" ht="62" customHeight="1" spans="2:24">
+      <c r="B137" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>775</v>
+      </c>
+      <c r="D137" s="3">
+        <v>46244.3541666667</v>
+      </c>
+      <c r="F137" s="119" t="s">
+        <v>776</v>
+      </c>
+      <c r="G137" s="119" t="s">
+        <v>777</v>
+      </c>
+      <c r="H137" s="119" t="s">
+        <v>778</v>
+      </c>
+      <c r="J137" s="119" t="s">
+        <v>779</v>
+      </c>
+      <c r="K137" s="119" t="s">
+        <v>780</v>
+      </c>
+      <c r="L137" s="119">
+        <v>14</v>
+      </c>
+      <c r="N137" s="41" t="s">
+        <v>781</v>
+      </c>
+      <c r="O137" s="42" t="s">
+        <v>782</v>
+      </c>
+      <c r="P137" s="42"/>
+      <c r="Q137" s="42"/>
+      <c r="R137" s="42"/>
+    </row>
+    <row r="138" s="5" customFormat="1" ht="53" spans="2:24">
+      <c r="B138" s="2" t="s">
+        <v>783</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="D138" s="2">
+        <v>1</v>
+      </c>
+      <c r="F138" s="61" t="s">
+        <v>518</v>
+      </c>
+      <c r="G138" s="61"/>
+      <c r="H138" s="61"/>
+      <c r="J138" s="119" t="s">
+        <v>785</v>
+      </c>
+      <c r="K138" s="119" t="s">
+        <v>786</v>
+      </c>
+      <c r="L138" s="119">
+        <v>99.5</v>
+      </c>
+      <c r="N138" s="51" t="s">
+        <v>787</v>
+      </c>
+      <c r="O138" s="51"/>
+      <c r="P138" s="51"/>
+    </row>
+    <row r="139" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="B139" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H139" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J139" s="119" t="s">
+        <v>789</v>
+      </c>
+      <c r="K139" s="119" t="s">
+        <v>790</v>
+      </c>
+      <c r="L139" s="119">
+        <v>88</v>
+      </c>
+      <c r="N139" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O139" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P139" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="140" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B140" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="F140" s="41" t="s">
+        <v>793</v>
+      </c>
+      <c r="G140" s="41" t="s">
+        <v>794</v>
+      </c>
+      <c r="H140" s="41" t="s">
+        <v>795</v>
+      </c>
+      <c r="J140" s="119" t="s">
+        <v>796</v>
+      </c>
+      <c r="K140" s="119" t="s">
+        <v>797</v>
+      </c>
+      <c r="L140" s="119">
+        <v>0.35</v>
+      </c>
+      <c r="N140" s="119" t="s">
+        <v>798</v>
+      </c>
+      <c r="O140" s="119" t="s">
+        <v>799</v>
+      </c>
+      <c r="P140" s="151">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="141" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B141" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="D141" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F141" s="41" t="s">
+        <v>802</v>
+      </c>
+      <c r="G141" s="41" t="s">
+        <v>803</v>
+      </c>
+      <c r="H141" s="41" t="s">
+        <v>692</v>
+      </c>
+      <c r="J141" s="119" t="s">
+        <v>804</v>
+      </c>
+      <c r="K141" s="119" t="s">
+        <v>805</v>
+      </c>
+      <c r="L141" s="119">
+        <v>0.1</v>
+      </c>
+      <c r="N141" s="119" t="s">
+        <v>806</v>
+      </c>
+      <c r="O141" s="119" t="s">
+        <v>807</v>
+      </c>
+      <c r="P141" s="151">
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="142" s="5" customFormat="1" ht="34" spans="2:24">
+      <c r="B142" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="D142" s="152">
+        <v>40</v>
+      </c>
+      <c r="J142" s="119" t="s">
+        <v>810</v>
+      </c>
+      <c r="K142" s="119" t="s">
+        <v>811</v>
+      </c>
+      <c r="L142" s="119">
+        <v>2</v>
+      </c>
+      <c r="N142" s="119" t="s">
+        <v>150</v>
+      </c>
+      <c r="O142" s="119" t="s">
+        <v>812</v>
+      </c>
+      <c r="P142" s="151">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="143" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B143" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="D143" s="2">
+        <v>4000</v>
+      </c>
+      <c r="J143" s="119" t="s">
+        <v>815</v>
+      </c>
+      <c r="K143" s="119" t="s">
+        <v>816</v>
+      </c>
+      <c r="L143" s="119" t="s">
+        <v>817</v>
+      </c>
+      <c r="N143" s="119" t="s">
+        <v>818</v>
+      </c>
+      <c r="O143" s="119" t="s">
+        <v>819</v>
+      </c>
+      <c r="P143" s="119">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="144" s="5" customFormat="1" ht="34" spans="2:24">
+      <c r="B144" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="D144" s="2">
+        <v>5000</v>
+      </c>
+      <c r="J144" s="119" t="s">
+        <v>822</v>
+      </c>
+      <c r="K144" s="119" t="s">
+        <v>129</v>
+      </c>
+      <c r="L144" s="119" t="s">
+        <v>130</v>
+      </c>
+      <c r="N144" s="119" t="s">
+        <v>164</v>
+      </c>
+      <c r="O144" s="119" t="s">
+        <v>823</v>
+      </c>
+      <c r="P144" s="151">
+        <v>162500</v>
+      </c>
+    </row>
+    <row r="145" s="5" customFormat="1" ht="36" spans="2:24">
+      <c r="B145" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="D145" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="J145" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="K145" s="119" t="s">
+        <v>231</v>
+      </c>
+      <c r="L145" s="119" t="s">
+        <v>445</v>
+      </c>
+      <c r="N145" s="119" t="s">
+        <v>220</v>
+      </c>
+      <c r="O145" s="119" t="s">
+        <v>826</v>
+      </c>
+      <c r="P145" s="151">
+        <v>3250</v>
+      </c>
+    </row>
+    <row r="146" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="B146" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="147" s="5" customFormat="1" ht="18" spans="2:24">
+      <c r="B147" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="F147" s="153" t="s">
+        <v>543</v>
+      </c>
+      <c r="G147" s="153" t="s">
+        <v>97</v>
+      </c>
+      <c r="H147" s="153" t="s">
+        <v>5</v>
+      </c>
+      <c r="I147" s="154" t="s">
+        <v>4</v>
+      </c>
+      <c r="J147" s="154"/>
+      <c r="K147" s="154"/>
+    </row>
+    <row r="148" s="5" customFormat="1" ht="36.75" spans="2:24">
+      <c r="B148" s="2" t="s">
+        <v>736</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="F148" s="100" t="s">
+        <v>831</v>
+      </c>
+      <c r="G148" s="100" t="s">
+        <v>740</v>
+      </c>
+      <c r="H148" s="21" t="s">
+        <v>741</v>
+      </c>
+      <c r="I148" s="155" t="s">
+        <v>742</v>
+      </c>
+      <c r="J148" s="155"/>
+      <c r="K148" s="155"/>
+    </row>
+    <row r="149" s="5" customFormat="1" ht="18.75" spans="2:24">
+      <c r="B149" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="D149" s="3">
+        <v>46244.4166666667</v>
+      </c>
+      <c r="F149" s="100" t="s">
+        <v>831</v>
+      </c>
+      <c r="G149" s="100" t="s">
+        <v>761</v>
+      </c>
+      <c r="H149" s="21" t="s">
+        <v>834</v>
+      </c>
+      <c r="I149" s="156">
+        <v>46231</v>
+      </c>
+      <c r="J149" s="156"/>
+      <c r="K149" s="156"/>
+    </row>
+    <row r="150" s="5" customFormat="1" ht="36.75" spans="2:24">
+      <c r="B150" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="D150" s="3">
+        <v>46244.375</v>
+      </c>
+      <c r="F150" s="100" t="s">
+        <v>831</v>
+      </c>
+      <c r="G150" s="100" t="s">
+        <v>764</v>
+      </c>
+      <c r="H150" s="21" t="s">
+        <v>765</v>
+      </c>
+      <c r="I150" s="155" t="s">
+        <v>766</v>
+      </c>
+      <c r="J150" s="155"/>
+      <c r="K150" s="155"/>
+    </row>
+    <row r="151" s="5" customFormat="1" ht="32" spans="2:24">
+      <c r="B151" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F151" s="100" t="s">
+        <v>838</v>
+      </c>
+      <c r="G151" s="100" t="s">
+        <v>839</v>
+      </c>
+      <c r="H151" s="21" t="s">
+        <v>840</v>
+      </c>
+      <c r="I151" s="155" t="s">
+        <v>841</v>
+      </c>
+      <c r="J151" s="155"/>
+      <c r="K151" s="155"/>
+    </row>
+    <row r="152" ht="36" spans="2:24">
+      <c r="B152" s="2" t="s">
+        <v>842</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="154" ht="24" customHeight="1" spans="2:24">
+      <c r="B154" s="157" t="s">
+        <v>844</v>
+      </c>
+      <c r="C154" s="157"/>
+      <c r="D154" s="157"/>
+      <c r="E154" s="157"/>
+      <c r="F154" s="157"/>
+      <c r="G154" s="157"/>
+      <c r="H154" s="157"/>
+      <c r="I154" s="157"/>
+      <c r="J154" s="157"/>
+      <c r="K154" s="157"/>
+      <c r="L154" s="157"/>
+      <c r="M154" s="157"/>
+      <c r="N154" s="157"/>
+      <c r="O154" s="157"/>
+      <c r="P154" s="157"/>
+      <c r="Q154" s="33"/>
+      <c r="R154" s="33"/>
+      <c r="S154" s="33"/>
+      <c r="T154" s="33"/>
+      <c r="U154" s="33"/>
+      <c r="V154" s="33"/>
+      <c r="W154" s="33"/>
+      <c r="X154" s="33"/>
+    </row>
+    <row r="155" ht="45" customHeight="1" spans="2:24">
+      <c r="B155" s="125" t="s">
+        <v>845</v>
+      </c>
+      <c r="C155" s="125"/>
+      <c r="D155" s="125"/>
+      <c r="E155" s="125"/>
+      <c r="F155" s="125"/>
+      <c r="G155" s="125"/>
+      <c r="H155" s="125"/>
+      <c r="I155" s="125"/>
+      <c r="J155" s="125"/>
+      <c r="K155" s="125"/>
+      <c r="L155" s="125"/>
+      <c r="M155" s="125"/>
+      <c r="N155" s="125"/>
+      <c r="O155" s="125"/>
+      <c r="P155" s="125"/>
+      <c r="Q155" s="158"/>
+      <c r="R155" s="158"/>
+      <c r="S155" s="158"/>
+      <c r="T155" s="158"/>
+      <c r="U155" s="158"/>
+      <c r="V155" s="158"/>
+      <c r="W155" s="158"/>
+      <c r="X155" s="158"/>
+    </row>
+    <row r="156" ht="20.4" spans="2:24">
+      <c r="B156" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C156" s="51"/>
+      <c r="D156" s="51"/>
+      <c r="F156" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="G156" s="51"/>
+      <c r="H156" s="51"/>
+      <c r="J156" s="51" t="s">
+        <v>846</v>
+      </c>
+      <c r="K156" s="51"/>
+      <c r="L156" s="51"/>
+      <c r="N156" s="51" t="s">
+        <v>94</v>
+      </c>
+      <c r="O156" s="51"/>
+      <c r="P156" s="51"/>
+    </row>
+    <row r="157" ht="18" spans="2:24">
+      <c r="B157" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G157" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H157" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J157" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K157" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L157" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N157" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O157" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P157" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="158" ht="51" spans="2:24">
+      <c r="B158" s="119" t="s">
+        <v>847</v>
+      </c>
+      <c r="C158" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="D158" s="119" t="s">
+        <v>848</v>
+      </c>
+      <c r="F158" s="119" t="s">
+        <v>849</v>
+      </c>
+      <c r="G158" s="119" t="s">
+        <v>850</v>
+      </c>
+      <c r="H158" s="119" t="s">
+        <v>739</v>
+      </c>
+      <c r="J158" s="119" t="s">
+        <v>851</v>
+      </c>
+      <c r="K158" s="119" t="s">
+        <v>852</v>
+      </c>
+      <c r="L158" s="151">
+        <v>162500</v>
+      </c>
+      <c r="N158" s="119" t="s">
+        <v>779</v>
+      </c>
+      <c r="O158" s="119" t="s">
+        <v>780</v>
+      </c>
+      <c r="P158" s="119">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="159" ht="34" spans="2:24">
+      <c r="B159" s="119" t="s">
+        <v>849</v>
+      </c>
+      <c r="C159" s="119" t="s">
+        <v>850</v>
+      </c>
+      <c r="D159" s="119" t="s">
+        <v>739</v>
+      </c>
+      <c r="J159" s="119" t="s">
+        <v>853</v>
+      </c>
+      <c r="K159" s="119" t="s">
+        <v>854</v>
+      </c>
+      <c r="L159" s="119">
+        <v>50</v>
+      </c>
+      <c r="N159" s="119" t="s">
+        <v>785</v>
+      </c>
+      <c r="O159" s="119" t="s">
+        <v>786</v>
+      </c>
+      <c r="P159" s="119">
+        <v>99.5</v>
+      </c>
+    </row>
+    <row r="160" ht="51" spans="2:24">
+      <c r="B160" s="119" t="s">
+        <v>855</v>
+      </c>
+      <c r="C160" s="119" t="s">
+        <v>856</v>
+      </c>
+      <c r="D160" s="119" t="s">
+        <v>748</v>
+      </c>
+      <c r="F160" s="61" t="s">
+        <v>518</v>
+      </c>
+      <c r="G160" s="61"/>
+      <c r="H160" s="61"/>
+      <c r="J160" s="119" t="s">
+        <v>220</v>
+      </c>
+      <c r="K160" s="119" t="s">
+        <v>857</v>
+      </c>
+      <c r="L160" s="151">
+        <v>3250</v>
+      </c>
+      <c r="N160" s="119" t="s">
+        <v>789</v>
+      </c>
+      <c r="O160" s="119" t="s">
+        <v>790</v>
+      </c>
+      <c r="P160" s="119">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="161" ht="34" spans="2:24">
+      <c r="B161" s="119" t="s">
+        <v>858</v>
+      </c>
+      <c r="C161" s="119" t="s">
+        <v>859</v>
+      </c>
+      <c r="D161" s="119" t="s">
+        <v>860</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G161" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H161" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J161" s="119" t="s">
+        <v>861</v>
+      </c>
+      <c r="K161" s="119" t="s">
+        <v>862</v>
+      </c>
+      <c r="L161" s="119">
+        <v>50</v>
+      </c>
+      <c r="N161" s="119" t="s">
+        <v>796</v>
+      </c>
+      <c r="O161" s="119" t="s">
+        <v>797</v>
+      </c>
+      <c r="P161" s="119">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="162" ht="34" spans="2:24">
+      <c r="B162" s="119" t="s">
+        <v>832</v>
+      </c>
+      <c r="C162" s="119" t="s">
+        <v>863</v>
+      </c>
+      <c r="D162" s="159">
+        <v>46244.4166666667</v>
+      </c>
+      <c r="F162" s="98" t="s">
+        <v>793</v>
+      </c>
+      <c r="G162" s="98" t="s">
+        <v>794</v>
+      </c>
+      <c r="H162" s="98" t="s">
+        <v>864</v>
+      </c>
+      <c r="J162" s="119" t="s">
+        <v>865</v>
+      </c>
+      <c r="K162" s="119" t="s">
+        <v>866</v>
+      </c>
+      <c r="L162" s="151">
+        <v>162500</v>
+      </c>
+      <c r="N162" s="119" t="s">
+        <v>804</v>
+      </c>
+      <c r="O162" s="119" t="s">
+        <v>805</v>
+      </c>
+      <c r="P162" s="119">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="163" ht="34" spans="2:24">
+      <c r="B163" s="119" t="s">
+        <v>867</v>
+      </c>
+      <c r="C163" s="119" t="s">
+        <v>868</v>
+      </c>
+      <c r="D163" s="160">
+        <v>2000</v>
+      </c>
+      <c r="F163" s="98" t="s">
+        <v>802</v>
+      </c>
+      <c r="G163" s="98" t="s">
+        <v>803</v>
+      </c>
+      <c r="H163" s="98" t="s">
+        <v>615</v>
+      </c>
+      <c r="J163" s="119" t="s">
+        <v>869</v>
+      </c>
+      <c r="K163" s="119" t="s">
+        <v>870</v>
+      </c>
+      <c r="L163" s="119">
+        <v>0</v>
+      </c>
+      <c r="N163" s="119" t="s">
+        <v>810</v>
+      </c>
+      <c r="O163" s="119" t="s">
+        <v>811</v>
+      </c>
+      <c r="P163" s="119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" ht="34" spans="2:24">
+      <c r="B164" s="119" t="s">
+        <v>853</v>
+      </c>
+      <c r="C164" s="119" t="s">
+        <v>871</v>
+      </c>
+      <c r="D164" s="119">
+        <v>50</v>
+      </c>
+      <c r="F164" s="161"/>
+      <c r="G164" s="161"/>
+      <c r="H164" s="161"/>
+      <c r="J164" s="119" t="s">
+        <v>872</v>
+      </c>
+      <c r="K164" s="119" t="s">
+        <v>873</v>
+      </c>
+      <c r="L164" s="119">
+        <v>0</v>
+      </c>
+      <c r="N164" s="119" t="s">
+        <v>815</v>
+      </c>
+      <c r="O164" s="119" t="s">
+        <v>816</v>
+      </c>
+      <c r="P164" s="119" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="165" ht="17" spans="2:24">
+      <c r="B165" s="119" t="s">
+        <v>874</v>
+      </c>
+      <c r="C165" s="119" t="s">
+        <v>875</v>
+      </c>
+      <c r="D165" s="119">
+        <v>500</v>
+      </c>
+      <c r="N165" s="119" t="s">
+        <v>822</v>
+      </c>
+      <c r="O165" s="119" t="s">
+        <v>129</v>
+      </c>
+      <c r="P165" s="119" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="166" ht="34" spans="2:24">
+      <c r="B166" s="119" t="s">
+        <v>869</v>
+      </c>
+      <c r="C166" s="119" t="s">
+        <v>876</v>
+      </c>
+      <c r="D166" s="119">
+        <v>12.5</v>
+      </c>
+      <c r="N166" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="O166" s="119" t="s">
+        <v>231</v>
+      </c>
+      <c r="P166" s="119" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="168" ht="20.4" spans="2:24">
+      <c r="B168" s="157" t="s">
+        <v>877</v>
+      </c>
+      <c r="C168" s="157"/>
+      <c r="D168" s="157"/>
+      <c r="E168" s="157"/>
+      <c r="F168" s="157"/>
+      <c r="G168" s="157"/>
+      <c r="H168" s="157"/>
+      <c r="I168" s="157"/>
+      <c r="J168" s="157"/>
+      <c r="K168" s="157"/>
+      <c r="L168" s="157"/>
+      <c r="M168" s="157"/>
+      <c r="N168" s="157"/>
+      <c r="O168" s="157"/>
+      <c r="P168" s="157"/>
+      <c r="Q168" s="33"/>
+      <c r="R168" s="33"/>
+      <c r="S168" s="33"/>
+      <c r="T168" s="33"/>
+      <c r="U168" s="33"/>
+      <c r="V168" s="33"/>
+      <c r="W168" s="33"/>
+      <c r="X168" s="33"/>
+    </row>
+    <row r="169" ht="52" customHeight="1" spans="2:24">
+      <c r="B169" s="162" t="s">
+        <v>878</v>
+      </c>
+      <c r="C169" s="162"/>
+      <c r="D169" s="162"/>
+      <c r="E169" s="162"/>
+      <c r="F169" s="162"/>
+      <c r="G169" s="162"/>
+      <c r="H169" s="162"/>
+      <c r="I169" s="162"/>
+      <c r="J169" s="162"/>
+      <c r="K169" s="162"/>
+      <c r="L169" s="162"/>
+      <c r="M169" s="162"/>
+      <c r="N169" s="162"/>
+      <c r="O169" s="162"/>
+      <c r="P169" s="162"/>
+      <c r="Q169" s="158"/>
+      <c r="R169" s="158"/>
+      <c r="S169" s="158"/>
+      <c r="T169" s="158"/>
+      <c r="U169" s="158"/>
+      <c r="V169" s="158"/>
+      <c r="W169" s="158"/>
+      <c r="X169" s="158"/>
+    </row>
+    <row r="170" ht="20.4" spans="2:24">
+      <c r="B170" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C170" s="51"/>
+      <c r="D170" s="51"/>
+      <c r="E170" s="163"/>
+      <c r="F170" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="G170" s="51"/>
+      <c r="H170" s="51"/>
+      <c r="I170" s="158"/>
+      <c r="J170" s="51" t="s">
+        <v>846</v>
+      </c>
+      <c r="K170" s="51"/>
+      <c r="L170" s="51"/>
+      <c r="M170" s="158"/>
+      <c r="N170" s="51" t="s">
+        <v>94</v>
+      </c>
+      <c r="O170" s="51"/>
+      <c r="P170" s="51"/>
+      <c r="Q170" s="158"/>
+      <c r="R170" s="158"/>
+      <c r="S170" s="158"/>
+      <c r="T170" s="158"/>
+      <c r="U170" s="158"/>
+      <c r="V170" s="158"/>
+      <c r="W170" s="158"/>
+      <c r="X170" s="158"/>
+    </row>
+    <row r="171" ht="18" spans="2:24">
+      <c r="B171" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D171" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G171" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H171" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J171" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K171" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L171" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N171" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O171" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P171" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="172" ht="51" spans="2:24">
+      <c r="B172" s="119" t="s">
+        <v>879</v>
+      </c>
+      <c r="C172" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="D172" s="119" t="s">
+        <v>795</v>
+      </c>
+      <c r="F172" s="119" t="s">
+        <v>849</v>
+      </c>
+      <c r="G172" s="119" t="s">
+        <v>850</v>
+      </c>
+      <c r="H172" s="119" t="s">
+        <v>739</v>
+      </c>
+      <c r="J172" s="119" t="s">
+        <v>880</v>
+      </c>
+      <c r="K172" s="119" t="s">
+        <v>881</v>
+      </c>
+      <c r="L172" s="151">
+        <v>162500</v>
+      </c>
+      <c r="N172" s="119" t="s">
+        <v>779</v>
+      </c>
+      <c r="O172" s="119" t="s">
+        <v>780</v>
+      </c>
+      <c r="P172" s="119">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="173" ht="34" spans="2:24">
+      <c r="B173" s="119" t="s">
+        <v>882</v>
+      </c>
+      <c r="C173" s="119" t="s">
+        <v>883</v>
+      </c>
+      <c r="D173" s="119" t="s">
+        <v>884</v>
+      </c>
+      <c r="J173" s="119" t="s">
+        <v>885</v>
+      </c>
+      <c r="K173" s="119" t="s">
+        <v>886</v>
+      </c>
+      <c r="L173" s="119">
+        <v>50</v>
+      </c>
+      <c r="N173" s="119" t="s">
+        <v>785</v>
+      </c>
+      <c r="O173" s="119" t="s">
+        <v>786</v>
+      </c>
+      <c r="P173" s="119">
+        <v>99.5</v>
+      </c>
+    </row>
+    <row r="174" ht="51" spans="2:24">
+      <c r="B174" s="119" t="s">
+        <v>849</v>
+      </c>
+      <c r="C174" s="119" t="s">
+        <v>850</v>
+      </c>
+      <c r="D174" s="119" t="s">
+        <v>887</v>
+      </c>
+      <c r="F174" s="61" t="s">
+        <v>518</v>
+      </c>
+      <c r="G174" s="61"/>
+      <c r="H174" s="61"/>
+      <c r="J174" s="119" t="s">
+        <v>220</v>
+      </c>
+      <c r="K174" s="119" t="s">
+        <v>888</v>
+      </c>
+      <c r="L174" s="151">
+        <v>3250</v>
+      </c>
+      <c r="N174" s="119" t="s">
+        <v>789</v>
+      </c>
+      <c r="O174" s="119" t="s">
+        <v>790</v>
+      </c>
+      <c r="P174" s="119">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="175" ht="34" spans="2:24">
+      <c r="B175" s="119" t="s">
+        <v>889</v>
+      </c>
+      <c r="C175" s="119" t="s">
+        <v>890</v>
+      </c>
+      <c r="D175" s="119" t="s">
+        <v>759</v>
+      </c>
+      <c r="F175" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G175" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H175" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J175" s="119" t="s">
+        <v>891</v>
+      </c>
+      <c r="K175" s="119" t="s">
+        <v>892</v>
+      </c>
+      <c r="L175" s="119">
+        <v>50</v>
+      </c>
+      <c r="N175" s="119" t="s">
+        <v>796</v>
+      </c>
+      <c r="O175" s="119" t="s">
+        <v>797</v>
+      </c>
+      <c r="P175" s="119">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="176" ht="34" spans="2:24">
+      <c r="B176" s="119" t="s">
+        <v>893</v>
+      </c>
+      <c r="C176" s="119" t="s">
+        <v>894</v>
+      </c>
+      <c r="D176" s="119" t="s">
+        <v>895</v>
+      </c>
+      <c r="F176" s="119" t="s">
+        <v>802</v>
+      </c>
+      <c r="G176" s="119" t="s">
+        <v>896</v>
+      </c>
+      <c r="H176" s="119" t="s">
+        <v>692</v>
+      </c>
+      <c r="J176" s="119" t="s">
+        <v>897</v>
+      </c>
+      <c r="K176" s="119" t="s">
+        <v>898</v>
+      </c>
+      <c r="L176" s="151">
+        <v>162500</v>
+      </c>
+      <c r="N176" s="119" t="s">
+        <v>804</v>
+      </c>
+      <c r="O176" s="119" t="s">
+        <v>805</v>
+      </c>
+      <c r="P176" s="119">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="177" ht="34" spans="2:18">
+      <c r="B177" s="119" t="s">
+        <v>899</v>
+      </c>
+      <c r="C177" s="119" t="s">
+        <v>900</v>
+      </c>
+      <c r="D177" s="159">
+        <v>46244.5833333333</v>
+      </c>
+      <c r="F177" s="119" t="s">
+        <v>901</v>
+      </c>
+      <c r="G177" s="119" t="s">
+        <v>892</v>
+      </c>
+      <c r="H177" s="119">
+        <v>12.5</v>
+      </c>
+      <c r="J177" s="119" t="s">
+        <v>902</v>
+      </c>
+      <c r="K177" s="119" t="s">
+        <v>903</v>
+      </c>
+      <c r="L177" s="119">
+        <v>0</v>
+      </c>
+      <c r="N177" s="119" t="s">
+        <v>810</v>
+      </c>
+      <c r="O177" s="119" t="s">
+        <v>811</v>
+      </c>
+      <c r="P177" s="119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="178" ht="34" spans="2:18">
+      <c r="B178" s="164" t="s">
+        <v>904</v>
+      </c>
+      <c r="C178" s="164" t="s">
+        <v>905</v>
+      </c>
+      <c r="D178" s="164">
+        <v>500</v>
+      </c>
+      <c r="F178" s="164" t="s">
+        <v>906</v>
+      </c>
+      <c r="G178" s="164" t="s">
+        <v>907</v>
+      </c>
+      <c r="H178" s="164">
+        <v>0</v>
+      </c>
+      <c r="J178" s="164" t="s">
+        <v>908</v>
+      </c>
+      <c r="K178" s="164" t="s">
+        <v>909</v>
+      </c>
+      <c r="L178" s="164">
+        <v>0</v>
+      </c>
+      <c r="N178" s="119" t="s">
+        <v>815</v>
+      </c>
+      <c r="O178" s="119" t="s">
+        <v>816</v>
+      </c>
+      <c r="P178" s="119" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="179" ht="20.4" spans="2:18">
+      <c r="B179" s="157" t="s">
+        <v>910</v>
+      </c>
+      <c r="C179" s="157"/>
+      <c r="D179" s="157"/>
+      <c r="E179" s="157"/>
+      <c r="F179" s="157"/>
+      <c r="G179" s="157"/>
+      <c r="H179" s="157"/>
+      <c r="I179" s="157"/>
+      <c r="J179" s="157"/>
+      <c r="K179" s="157"/>
+      <c r="L179" s="157"/>
+      <c r="N179" s="119" t="s">
+        <v>822</v>
+      </c>
+      <c r="O179" s="119" t="s">
+        <v>129</v>
+      </c>
+      <c r="P179" s="119" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="180" ht="34" spans="2:18">
+      <c r="B180" s="165" t="s">
+        <v>0</v>
+      </c>
+      <c r="C180" s="166" t="s">
+        <v>911</v>
+      </c>
+      <c r="D180" s="166"/>
+      <c r="E180" s="167"/>
+      <c r="F180" s="166" t="s">
+        <v>912</v>
+      </c>
+      <c r="G180" s="166"/>
+      <c r="H180" s="166"/>
+      <c r="I180" s="167"/>
+      <c r="J180" s="168" t="s">
+        <v>913</v>
+      </c>
+      <c r="K180" s="168"/>
+      <c r="L180" s="168"/>
+      <c r="N180" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="O180" s="119" t="s">
+        <v>231</v>
+      </c>
+      <c r="P180" s="119" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="181" ht="34" spans="2:18">
+      <c r="B181" s="41" t="s">
+        <v>914</v>
+      </c>
+      <c r="C181" s="133" t="s">
+        <v>823</v>
+      </c>
+      <c r="D181" s="133"/>
+      <c r="F181" s="133" t="s">
+        <v>826</v>
+      </c>
+      <c r="G181" s="133"/>
+      <c r="H181" s="133"/>
+      <c r="J181" s="119" t="s">
+        <v>872</v>
+      </c>
+      <c r="K181" s="119" t="s">
+        <v>873</v>
+      </c>
+      <c r="L181" s="119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" ht="36" spans="2:18">
+      <c r="B182" s="41" t="s">
+        <v>915</v>
+      </c>
+      <c r="C182" s="133" t="s">
+        <v>916</v>
+      </c>
+      <c r="D182" s="133"/>
+      <c r="F182" s="133" t="s">
+        <v>857</v>
+      </c>
+      <c r="G182" s="133"/>
+      <c r="H182" s="133"/>
+    </row>
+    <row r="183" ht="36" spans="2:18">
+      <c r="B183" s="41" t="s">
+        <v>917</v>
+      </c>
+      <c r="C183" s="133" t="s">
+        <v>918</v>
+      </c>
+      <c r="D183" s="133"/>
+      <c r="F183" s="133" t="s">
+        <v>888</v>
+      </c>
+      <c r="G183" s="133"/>
+      <c r="H183" s="133"/>
+    </row>
+    <row r="184" ht="9" customHeight="1"/>
+    <row r="185" ht="31" customHeight="1" spans="2:18">
+      <c r="B185" s="6" t="s">
+        <v>919</v>
+      </c>
+      <c r="C185" s="6"/>
+      <c r="D185" s="6"/>
+      <c r="E185" s="6"/>
+      <c r="F185" s="6"/>
+      <c r="G185" s="6"/>
+      <c r="H185" s="6"/>
+      <c r="I185" s="6"/>
+      <c r="J185" s="6"/>
+      <c r="K185" s="6"/>
+      <c r="L185" s="6"/>
+      <c r="M185" s="6"/>
+      <c r="N185" s="6"/>
+      <c r="O185" s="6"/>
+      <c r="P185" s="6"/>
+      <c r="Q185" s="33"/>
+      <c r="R185" s="33"/>
+    </row>
+    <row r="186" ht="63" customHeight="1" spans="2:18">
+      <c r="B186" s="169" t="s">
+        <v>920</v>
+      </c>
+      <c r="C186" s="169"/>
+      <c r="D186" s="169"/>
+      <c r="E186" s="169"/>
+      <c r="F186" s="169"/>
+      <c r="G186" s="169"/>
+      <c r="H186" s="169"/>
+      <c r="I186" s="169"/>
+      <c r="J186" s="169"/>
+      <c r="K186" s="169"/>
+      <c r="L186" s="169"/>
+      <c r="M186" s="169"/>
+      <c r="N186" s="169"/>
+      <c r="O186" s="169"/>
+      <c r="P186" s="169"/>
+    </row>
+    <row r="187" ht="20.4" spans="2:18">
+      <c r="B187" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C187" s="51"/>
+      <c r="D187" s="51"/>
+      <c r="F187" s="51" t="s">
+        <v>921</v>
+      </c>
+      <c r="G187" s="51"/>
+      <c r="H187" s="51"/>
+      <c r="J187" s="51" t="s">
+        <v>922</v>
+      </c>
+      <c r="K187" s="51"/>
+      <c r="L187" s="51"/>
+      <c r="N187" s="51" t="s">
+        <v>344</v>
+      </c>
+      <c r="O187" s="51"/>
+      <c r="P187" s="51"/>
+    </row>
+    <row r="188" ht="18" spans="2:18">
+      <c r="B188" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D188" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F188" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G188" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H188" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J188" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K188" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L188" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N188" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O188" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P188" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="189" ht="53" spans="2:18">
+      <c r="B189" s="119" t="s">
+        <v>740</v>
+      </c>
+      <c r="C189" s="119" t="s">
+        <v>923</v>
+      </c>
+      <c r="D189" s="119" t="s">
+        <v>742</v>
+      </c>
+      <c r="F189" s="119" t="s">
+        <v>779</v>
+      </c>
+      <c r="G189" s="119" t="s">
+        <v>924</v>
+      </c>
+      <c r="H189" s="119">
+        <v>14</v>
+      </c>
+      <c r="J189" s="41" t="s">
+        <v>849</v>
+      </c>
+      <c r="K189" s="41" t="s">
+        <v>925</v>
+      </c>
+      <c r="L189" s="41" t="s">
+        <v>887</v>
+      </c>
+      <c r="N189" s="98" t="s">
+        <v>926</v>
+      </c>
+      <c r="O189" s="98" t="s">
+        <v>927</v>
+      </c>
+      <c r="P189" s="98" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="190" ht="34" spans="2:18">
+      <c r="B190" s="119" t="s">
+        <v>753</v>
+      </c>
+      <c r="C190" s="119" t="s">
+        <v>754</v>
+      </c>
+      <c r="D190" s="119" t="s">
+        <v>755</v>
+      </c>
+      <c r="F190" s="119" t="s">
+        <v>785</v>
+      </c>
+      <c r="G190" s="119" t="s">
+        <v>929</v>
+      </c>
+      <c r="H190" s="119">
+        <v>99.5</v>
+      </c>
+      <c r="N190" s="98" t="s">
+        <v>379</v>
+      </c>
+      <c r="O190" s="98" t="s">
+        <v>575</v>
+      </c>
+      <c r="P190" s="98" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="191" ht="34" spans="2:18">
+      <c r="B191" s="119" t="s">
+        <v>930</v>
+      </c>
+      <c r="C191" s="119" t="s">
+        <v>931</v>
+      </c>
+      <c r="D191" s="119" t="s">
+        <v>932</v>
+      </c>
+      <c r="F191" s="119" t="s">
+        <v>789</v>
+      </c>
+      <c r="G191" s="119" t="s">
+        <v>933</v>
+      </c>
+      <c r="H191" s="119">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="192" ht="34" spans="2:18">
+      <c r="B192" s="119" t="s">
+        <v>791</v>
+      </c>
+      <c r="C192" s="119" t="s">
+        <v>792</v>
+      </c>
+      <c r="D192" s="119" t="s">
+        <v>792</v>
+      </c>
+      <c r="F192" s="119" t="s">
+        <v>796</v>
+      </c>
+      <c r="G192" s="119" t="s">
+        <v>934</v>
+      </c>
+      <c r="H192" s="119">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="193" ht="34" spans="2:8">
+      <c r="B193" s="119" t="s">
+        <v>935</v>
+      </c>
+      <c r="C193" s="119" t="s">
+        <v>936</v>
+      </c>
+      <c r="D193" s="119" t="s">
+        <v>937</v>
+      </c>
+      <c r="F193" s="119" t="s">
+        <v>804</v>
+      </c>
+      <c r="G193" s="119" t="s">
+        <v>938</v>
+      </c>
+      <c r="H193" s="119">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="194" ht="34" spans="2:8">
+      <c r="B194" s="119" t="s">
+        <v>939</v>
+      </c>
+      <c r="C194" s="119" t="s">
+        <v>940</v>
+      </c>
+      <c r="D194" s="149">
+        <v>46231</v>
+      </c>
+      <c r="F194" s="119" t="s">
+        <v>810</v>
+      </c>
+      <c r="G194" s="119" t="s">
+        <v>941</v>
+      </c>
+      <c r="H194" s="119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="195" ht="34" spans="2:8">
+      <c r="B195" s="119" t="s">
+        <v>942</v>
+      </c>
+      <c r="C195" s="119" t="s">
+        <v>943</v>
+      </c>
+      <c r="D195" s="119" t="s">
+        <v>944</v>
+      </c>
+      <c r="F195" s="119" t="s">
+        <v>815</v>
+      </c>
+      <c r="G195" s="119" t="s">
+        <v>945</v>
+      </c>
+      <c r="H195" s="119" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="196" ht="17" spans="2:8">
+      <c r="B196" s="119" t="s">
+        <v>800</v>
+      </c>
+      <c r="C196" s="119" t="s">
+        <v>801</v>
+      </c>
+      <c r="D196" s="119">
+        <v>25</v>
+      </c>
+      <c r="F196" s="119" t="s">
+        <v>770</v>
+      </c>
+      <c r="G196" s="119" t="s">
+        <v>129</v>
+      </c>
+      <c r="H196" s="119" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="197" ht="34" spans="2:8">
+      <c r="B197" s="119" t="s">
+        <v>808</v>
+      </c>
+      <c r="C197" s="119" t="s">
+        <v>946</v>
+      </c>
+      <c r="D197" s="160">
+        <v>2000</v>
+      </c>
+      <c r="F197" s="119" t="s">
+        <v>764</v>
+      </c>
+      <c r="G197" s="119" t="s">
+        <v>947</v>
+      </c>
+      <c r="H197" s="119" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="198" ht="17" spans="2:8">
+      <c r="B198" s="119" t="s">
+        <v>813</v>
+      </c>
+      <c r="C198" s="119" t="s">
+        <v>948</v>
+      </c>
+      <c r="D198" s="119">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="200" spans="2:8">
+      <c r="B200" s="170" t="s">
+        <v>949</v>
+      </c>
+      <c r="C200" s="171"/>
+      <c r="D200" s="171"/>
+      <c r="F200" s="172" t="s">
+        <v>950</v>
+      </c>
+      <c r="G200" s="173"/>
+      <c r="H200" s="173"/>
+    </row>
+    <row r="201" spans="2:8">
+      <c r="B201" s="171"/>
+      <c r="C201" s="171"/>
+      <c r="D201" s="171"/>
+      <c r="F201" s="173"/>
+      <c r="G201" s="173"/>
+      <c r="H201" s="173"/>
+    </row>
+    <row r="202" spans="2:8">
+      <c r="B202" s="171"/>
+      <c r="C202" s="171"/>
+      <c r="D202" s="171"/>
+      <c r="F202" s="173"/>
+      <c r="G202" s="173"/>
+      <c r="H202" s="173"/>
+    </row>
+    <row r="203" spans="2:8">
+      <c r="B203" s="171"/>
+      <c r="C203" s="171"/>
+      <c r="D203" s="171"/>
+      <c r="F203" s="173"/>
+      <c r="G203" s="173"/>
+      <c r="H203" s="173"/>
+    </row>
+    <row r="204" spans="2:8">
+      <c r="B204" s="171"/>
+      <c r="C204" s="171"/>
+      <c r="D204" s="171"/>
+      <c r="F204" s="173"/>
+      <c r="G204" s="173"/>
+      <c r="H204" s="173"/>
+    </row>
+    <row r="205" spans="2:8">
+      <c r="B205" s="171"/>
+      <c r="C205" s="171"/>
+      <c r="D205" s="171"/>
+      <c r="F205" s="173"/>
+      <c r="G205" s="173"/>
+      <c r="H205" s="173"/>
+    </row>
+    <row r="206" spans="2:8">
+      <c r="B206" s="171"/>
+      <c r="C206" s="171"/>
+      <c r="D206" s="171"/>
+      <c r="F206" s="173"/>
+      <c r="G206" s="173"/>
+      <c r="H206" s="173"/>
+    </row>
+    <row r="207" spans="2:8">
+      <c r="B207" s="171"/>
+      <c r="C207" s="171"/>
+      <c r="D207" s="171"/>
+      <c r="F207" s="173"/>
+      <c r="G207" s="173"/>
+      <c r="H207" s="173"/>
+    </row>
   </sheetData>
-  <mergeCells count="157">
+  <mergeCells count="220">
     <mergeCell ref="B1:AB1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:H2"/>
@@ -10202,14 +13353,77 @@
     <mergeCell ref="B113:X113"/>
     <mergeCell ref="B114:D114"/>
     <mergeCell ref="F114:H114"/>
-    <mergeCell ref="F120:H120"/>
-    <mergeCell ref="G121:H121"/>
-    <mergeCell ref="G122:H122"/>
-    <mergeCell ref="G123:H123"/>
+    <mergeCell ref="J114:L114"/>
+    <mergeCell ref="N114:P114"/>
+    <mergeCell ref="R114:T114"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="F121:H121"/>
+    <mergeCell ref="J121:P121"/>
+    <mergeCell ref="C122:D122"/>
+    <mergeCell ref="K122:P122"/>
+    <mergeCell ref="C123:D123"/>
+    <mergeCell ref="K123:P123"/>
+    <mergeCell ref="C124:D124"/>
+    <mergeCell ref="K124:P124"/>
+    <mergeCell ref="K125:P125"/>
+    <mergeCell ref="K126:P126"/>
+    <mergeCell ref="B128:R128"/>
+    <mergeCell ref="B129:R129"/>
+    <mergeCell ref="B130:D130"/>
+    <mergeCell ref="F130:H130"/>
+    <mergeCell ref="J130:L130"/>
+    <mergeCell ref="N130:R130"/>
+    <mergeCell ref="Q131:R131"/>
+    <mergeCell ref="Q132:R132"/>
+    <mergeCell ref="Q133:R133"/>
+    <mergeCell ref="N134:R134"/>
+    <mergeCell ref="J135:L135"/>
+    <mergeCell ref="O135:R135"/>
+    <mergeCell ref="O136:R136"/>
+    <mergeCell ref="O137:R137"/>
+    <mergeCell ref="F138:H138"/>
+    <mergeCell ref="N138:P138"/>
+    <mergeCell ref="I147:K147"/>
+    <mergeCell ref="I148:K148"/>
+    <mergeCell ref="I149:K149"/>
+    <mergeCell ref="I150:K150"/>
+    <mergeCell ref="I151:K151"/>
+    <mergeCell ref="B154:P154"/>
+    <mergeCell ref="B155:P155"/>
+    <mergeCell ref="B156:D156"/>
+    <mergeCell ref="F156:H156"/>
+    <mergeCell ref="J156:L156"/>
+    <mergeCell ref="N156:P156"/>
+    <mergeCell ref="F160:H160"/>
+    <mergeCell ref="B168:P168"/>
+    <mergeCell ref="B169:P169"/>
+    <mergeCell ref="B170:D170"/>
+    <mergeCell ref="F170:H170"/>
+    <mergeCell ref="J170:L170"/>
+    <mergeCell ref="N170:P170"/>
+    <mergeCell ref="F174:H174"/>
+    <mergeCell ref="B179:L179"/>
+    <mergeCell ref="C180:D180"/>
+    <mergeCell ref="F180:H180"/>
+    <mergeCell ref="J180:L180"/>
+    <mergeCell ref="C181:D181"/>
+    <mergeCell ref="F181:H181"/>
+    <mergeCell ref="C182:D182"/>
+    <mergeCell ref="F182:H182"/>
+    <mergeCell ref="C183:D183"/>
+    <mergeCell ref="F183:H183"/>
+    <mergeCell ref="B185:P185"/>
+    <mergeCell ref="B186:P186"/>
+    <mergeCell ref="B187:D187"/>
+    <mergeCell ref="F187:H187"/>
+    <mergeCell ref="J187:L187"/>
+    <mergeCell ref="N187:P187"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="K36:K38"/>
     <mergeCell ref="L36:L38"/>
     <mergeCell ref="W36:W38"/>
+    <mergeCell ref="B200:D207"/>
+    <mergeCell ref="F200:H207"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -10229,7 +13443,7 @@
   <sheetData>
     <row r="1" ht="409.5" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>707</v>
+        <v>951</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10278,6 +13492,27 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8"/>
+  <cols>
+    <col min="1" max="1" width="30.9230769230769" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1">
+        <f>3550000/1500</f>
+        <v>2366.66666666667</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>